<commit_message>
Update experiment results workbook
</commit_message>
<xml_diff>
--- a/results/experiment_results.xlsx
+++ b/results/experiment_results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a162c8629e60ce6/文档/工作二/实验/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\CodexPlace\Paper\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{D9F6B51C-1331-4E4E-9C7D-89742E410276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BDBE5E8-67D4-4C71-AC85-F9CD4E654937}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85960186-35E2-4BDD-8FF3-0550B6840645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="4056" windowWidth="23256" windowHeight="13176" xr2:uid="{A48CE7DE-C994-4FF0-933D-7A6BBA2A096A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A48CE7DE-C994-4FF0-933D-7A6BBA2A096A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="24">
   <si>
     <t>AVG</t>
   </si>
@@ -128,7 +128,7 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>0..289</t>
+    <t>Traffic</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -142,7 +142,7 @@
     <numFmt numFmtId="178" formatCode="0.000"/>
     <numFmt numFmtId="179" formatCode="0.000_ "/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,7 +617,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C92DFD3-BCDC-4725-8E66-D920EBEA03F0}">
   <dimension ref="A1:Z47"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="3"/>
     <col min="2" max="2" width="19" style="3" customWidth="1"/>
@@ -626,7 +626,7 @@
     <col min="6" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="G1" s="11" t="s">
         <v>13</v>
       </c>
@@ -668,7 +668,7 @@
       </c>
       <c r="Z1" s="11"/>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -742,7 +742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -824,7 +824,7 @@
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="11"/>
       <c r="B4" s="1">
         <v>192</v>
@@ -904,7 +904,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="11"/>
       <c r="B5" s="1">
         <v>336</v>
@@ -984,7 +984,7 @@
         <v>0.46500000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="11"/>
       <c r="B6" s="1">
         <v>720</v>
@@ -1064,7 +1064,7 @@
         <v>0.50700000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="11"/>
       <c r="B7" s="4" t="s">
         <v>0</v>
@@ -1092,6 +1092,12 @@
       <c r="H7" s="3">
         <v>0.42299999999999999</v>
       </c>
+      <c r="I7" s="3">
+        <v>0.439</v>
+      </c>
+      <c r="J7" s="3">
+        <v>0.437</v>
+      </c>
       <c r="K7" s="3">
         <v>0.42199999999999999</v>
       </c>
@@ -1141,7 +1147,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>6</v>
       </c>
@@ -1223,7 +1229,7 @@
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="11"/>
       <c r="B9" s="1">
         <v>192</v>
@@ -1303,7 +1309,7 @@
         <v>0.441</v>
       </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="11"/>
       <c r="B10" s="1">
         <v>336</v>
@@ -1383,7 +1389,7 @@
         <v>0.45900000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="11"/>
       <c r="B11" s="1">
         <v>720</v>
@@ -1463,7 +1469,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="11"/>
       <c r="B12" s="4" t="s">
         <v>0</v>
@@ -1484,6 +1490,18 @@
         <f t="shared" si="1"/>
         <v>0.38800000000000001</v>
       </c>
+      <c r="G12" s="3">
+        <v>0.38</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0.379</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0.38300000000000001</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0.39600000000000002</v>
+      </c>
       <c r="K12" s="3">
         <v>0.38100000000000001</v>
       </c>
@@ -1533,7 +1551,7 @@
         <v>0.45200000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="15">
+    <row r="13" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>7</v>
       </c>
@@ -1554,8 +1572,8 @@
         <f t="shared" si="1"/>
         <v>0.34599999999999997</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>23</v>
+      <c r="G13" s="3">
+        <v>0.28899999999999998</v>
       </c>
       <c r="H13" s="3">
         <v>0.33400000000000002</v>
@@ -1615,7 +1633,7 @@
         <v>0.39700000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="15">
+    <row r="14" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="11"/>
       <c r="B14" s="1">
         <v>192</v>
@@ -1695,7 +1713,7 @@
         <v>0.439</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="15">
+    <row r="15" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="11"/>
       <c r="B15" s="1">
         <v>336</v>
@@ -1775,7 +1793,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="15">
+    <row r="16" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="11"/>
       <c r="B16" s="1">
         <v>720</v>
@@ -1855,7 +1873,7 @@
         <v>0.47399999999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="15">
+    <row r="17" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
       <c r="B17" s="4" t="s">
         <v>0</v>
@@ -1876,6 +1894,18 @@
         <f t="shared" si="1"/>
         <v>0.38700000000000001</v>
       </c>
+      <c r="G17" s="3">
+        <v>0.373</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0.38</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0.40300000000000002</v>
+      </c>
       <c r="K17" s="3">
         <v>0.35299999999999998</v>
       </c>
@@ -1925,7 +1955,7 @@
         <v>0.44900000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:26">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>8</v>
       </c>
@@ -2007,7 +2037,7 @@
         <v>0.28699999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:26">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A19" s="11"/>
       <c r="B19" s="1">
         <v>192</v>
@@ -2087,7 +2117,7 @@
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:26">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A20" s="11"/>
       <c r="B20" s="1">
         <v>336</v>
@@ -2167,7 +2197,7 @@
         <v>0.36599999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:26">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A21" s="11"/>
       <c r="B21" s="1">
         <v>720</v>
@@ -2247,7 +2277,7 @@
         <v>0.41499999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:26">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A22" s="11"/>
       <c r="B22" s="4" t="s">
         <v>0</v>
@@ -2268,6 +2298,18 @@
         <f t="shared" si="1"/>
         <v>0.315</v>
       </c>
+      <c r="G22" s="3">
+        <v>0.27</v>
+      </c>
+      <c r="H22" s="3">
+        <v>0.312</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="J22" s="3">
+        <v>0.32700000000000001</v>
+      </c>
       <c r="K22" s="3">
         <v>0.27500000000000002</v>
       </c>
@@ -2317,7 +2359,7 @@
         <v>0.34899999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:26">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>9</v>
       </c>
@@ -2345,10 +2387,10 @@
         <v>0.219</v>
       </c>
       <c r="I23" s="3">
-        <v>0.14299999999999999</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="J23" s="3">
-        <v>0.23499999999999999</v>
+        <v>0.22900000000000001</v>
       </c>
       <c r="K23" s="3">
         <v>0.14099999999999999</v>
@@ -2399,7 +2441,7 @@
         <v>0.308</v>
       </c>
     </row>
-    <row r="24" spans="1:26">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A24" s="11"/>
       <c r="B24" s="1">
         <v>192</v>
@@ -2425,10 +2467,10 @@
         <v>0.23699999999999999</v>
       </c>
       <c r="I24" s="3">
-        <v>0.159</v>
+        <v>0.151</v>
       </c>
       <c r="J24" s="3">
-        <v>0.25</v>
+        <v>0.246</v>
       </c>
       <c r="K24" s="3">
         <v>0.151</v>
@@ -2479,7 +2521,7 @@
         <v>0.315</v>
       </c>
     </row>
-    <row r="25" spans="1:26">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A25" s="11"/>
       <c r="B25" s="1">
         <v>336</v>
@@ -2505,10 +2547,10 @@
         <v>0.255</v>
       </c>
       <c r="I25" s="3">
-        <v>0.17399999999999999</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="J25" s="3">
-        <v>0.26700000000000002</v>
+        <v>0.26800000000000002</v>
       </c>
       <c r="K25" s="3">
         <v>0.17299999999999999</v>
@@ -2559,7 +2601,7 @@
         <v>0.32900000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:26">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
       <c r="B26" s="1">
         <v>720</v>
@@ -2585,10 +2627,10 @@
         <v>0.27400000000000002</v>
       </c>
       <c r="I26" s="3">
-        <v>0.20300000000000001</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="J26" s="3">
-        <v>0.29299999999999998</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="K26" s="3">
         <v>0.20100000000000001</v>
@@ -2639,7 +2681,7 @@
         <v>0.35499999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:26">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A27" s="11"/>
       <c r="B27" s="4" t="s">
         <v>0</v>
@@ -2660,6 +2702,18 @@
         <f t="shared" si="1"/>
         <v>0.252</v>
       </c>
+      <c r="G27" s="3">
+        <v>0.158</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0.246</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0.16600000000000001</v>
+      </c>
+      <c r="J27" s="3">
+        <v>0.25900000000000001</v>
+      </c>
       <c r="K27" s="3">
         <v>0.16600000000000001</v>
       </c>
@@ -2709,7 +2763,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:26">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>10</v>
       </c>
@@ -2737,10 +2791,10 @@
         <v>0.19</v>
       </c>
       <c r="I28" s="3">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="J28" s="3">
-        <v>0.20699999999999999</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="K28" s="3">
         <v>0.16200000000000001</v>
@@ -2791,7 +2845,7 @@
         <v>0.29599999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:26">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A29" s="11"/>
       <c r="B29" s="1">
         <v>192</v>
@@ -2817,10 +2871,10 @@
         <v>0.23899999999999999</v>
       </c>
       <c r="I29" s="3">
-        <v>0.22</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="J29" s="3">
-        <v>0.254</v>
+        <v>0.25</v>
       </c>
       <c r="K29" s="3">
         <v>0.20799999999999999</v>
@@ -2871,7 +2925,7 @@
         <v>0.33600000000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:26">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A30" s="11"/>
       <c r="B30" s="1">
         <v>336</v>
@@ -2897,10 +2951,10 @@
         <v>0.28199999999999997</v>
       </c>
       <c r="I30" s="3">
-        <v>0.28199999999999997</v>
+        <v>0.26900000000000002</v>
       </c>
       <c r="J30" s="3">
-        <v>0.3</v>
+        <v>0.29599999999999999</v>
       </c>
       <c r="K30" s="3">
         <v>0.26300000000000001</v>
@@ -2951,7 +3005,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="31" spans="1:26">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A31" s="11"/>
       <c r="B31" s="1">
         <v>720</v>
@@ -2977,10 +3031,10 @@
         <v>0.33600000000000002</v>
       </c>
       <c r="I31" s="3">
-        <v>0.35699999999999998</v>
+        <v>0.34300000000000003</v>
       </c>
       <c r="J31" s="3">
-        <v>0.34899999999999998</v>
+        <v>0.33400000000000002</v>
       </c>
       <c r="K31" s="3">
         <v>0.34</v>
@@ -3031,7 +3085,7 @@
         <v>0.42799999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:26">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A32" s="11"/>
       <c r="B32" s="4" t="s">
         <v>0</v>
@@ -3052,6 +3106,18 @@
         <f t="shared" si="1"/>
         <v>0.26400000000000001</v>
       </c>
+      <c r="G32" s="3">
+        <v>0.24</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0.245</v>
+      </c>
+      <c r="J32" s="3">
+        <v>0.27100000000000002</v>
+      </c>
       <c r="K32" s="3">
         <v>0.24299999999999999</v>
       </c>
@@ -3101,7 +3167,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="33" spans="1:26">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>11</v>
       </c>
@@ -3129,10 +3195,10 @@
         <v>0.2</v>
       </c>
       <c r="I33" s="3">
-        <v>0.20499999999999999</v>
+        <v>0.192</v>
       </c>
       <c r="J33" s="3">
-        <v>0.23699999999999999</v>
+        <v>0.222</v>
       </c>
       <c r="K33" s="3">
         <v>0.16300000000000001</v>
@@ -3183,7 +3249,7 @@
         <v>0.34200000000000003</v>
       </c>
     </row>
-    <row r="34" spans="1:26">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A34" s="11"/>
       <c r="B34" s="1">
         <v>192</v>
@@ -3209,10 +3275,10 @@
         <v>0.22</v>
       </c>
       <c r="I34" s="3">
-        <v>0.22500000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="J34" s="3">
-        <v>0.248</v>
+        <v>0.251</v>
       </c>
       <c r="K34" s="3">
         <v>0.182</v>
@@ -3263,7 +3329,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="35" spans="1:26">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A35" s="11"/>
       <c r="B35" s="1">
         <v>336</v>
@@ -3289,7 +3355,7 @@
         <v>0.23100000000000001</v>
       </c>
       <c r="I35" s="3">
-        <v>0.246</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="J35" s="3">
         <v>0.26300000000000001</v>
@@ -3343,7 +3409,7 @@
         <v>0.376</v>
       </c>
     </row>
-    <row r="36" spans="1:26">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A36" s="11"/>
       <c r="B36" s="1">
         <v>720</v>
@@ -3369,10 +3435,10 @@
         <v>0.24299999999999999</v>
       </c>
       <c r="I36" s="3">
-        <v>0.878</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="J36" s="3">
-        <v>0.71499999999999997</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="K36" s="3">
         <v>0.19900000000000001</v>
@@ -3423,7 +3489,7 @@
         <v>0.42699999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:26">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A37" s="11"/>
       <c r="B37" s="4" t="s">
         <v>0</v>
@@ -3444,12 +3510,30 @@
         <f t="shared" si="1"/>
         <v>0.246</v>
       </c>
+      <c r="G37" s="3">
+        <v>0.19700000000000001</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0.224</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0.22700000000000001</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0.25</v>
+      </c>
       <c r="K37" s="3">
         <v>0.184</v>
       </c>
       <c r="L37" s="3">
         <v>0.247</v>
       </c>
+      <c r="M37" s="3">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="N37" s="3">
+        <v>0.255</v>
+      </c>
       <c r="O37" s="3">
         <v>0.23899999999999999</v>
       </c>
@@ -3487,7 +3571,7 @@
         <v>0.38100000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:26">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>12</v>
       </c>
@@ -3563,7 +3647,7 @@
         <v>0.28399999999999997</v>
       </c>
     </row>
-    <row r="39" spans="1:26">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A39" s="11"/>
       <c r="B39" s="1">
         <v>192</v>
@@ -3637,7 +3721,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="40" spans="1:26">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A40" s="11"/>
       <c r="B40" s="1">
         <v>336</v>
@@ -3711,7 +3795,7 @@
         <v>0.51100000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:26">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A41" s="11"/>
       <c r="B41" s="1">
         <v>720</v>
@@ -3785,7 +3869,7 @@
         <v>0.83199999999999996</v>
       </c>
     </row>
-    <row r="42" spans="1:26">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A42" s="11"/>
       <c r="B42" s="4" t="s">
         <v>0</v>
@@ -3806,6 +3890,18 @@
         <f t="shared" si="1"/>
         <v>0.39700000000000002</v>
       </c>
+      <c r="G42" s="3">
+        <v>0.35499999999999998</v>
+      </c>
+      <c r="H42" s="3">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="K42" s="3">
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="L42" s="3">
+        <v>0.40799999999999997</v>
+      </c>
       <c r="M42" s="3">
         <v>0.35199999999999998</v>
       </c>
@@ -3849,7 +3945,25 @@
         <v>0.51100000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:26">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A43" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B43" s="1">
+        <v>96</v>
+      </c>
+      <c r="C43" s="3">
+        <v>0.40793699999999999</v>
+      </c>
+      <c r="D43" s="3">
+        <v>0.40699999999999997</v>
+      </c>
+      <c r="E43" s="3">
+        <v>0.261187</v>
+      </c>
+      <c r="F43" s="3">
+        <v>0.26100000000000001</v>
+      </c>
       <c r="G43" s="3">
         <v>0.4</v>
       </c>
@@ -3857,10 +3971,10 @@
         <v>0.23699999999999999</v>
       </c>
       <c r="I43" s="3">
-        <v>0.51200000000000001</v>
+        <v>0.38600000000000001</v>
       </c>
       <c r="J43" s="3">
-        <v>0.35399999999999998</v>
+        <v>0.25800000000000001</v>
       </c>
       <c r="K43" s="3">
         <v>0.41</v>
@@ -3911,7 +4025,23 @@
         <v>0.36599999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:26">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A44" s="11"/>
+      <c r="B44" s="1">
+        <v>192</v>
+      </c>
+      <c r="C44" s="3">
+        <v>0.42424499999999998</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0.42399999999999999</v>
+      </c>
+      <c r="E44" s="3">
+        <v>0.26533000000000001</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0.26500000000000001</v>
+      </c>
       <c r="G44" s="3">
         <v>0.41799999999999998</v>
       </c>
@@ -3973,7 +4103,23 @@
         <v>0.373</v>
       </c>
     </row>
-    <row r="45" spans="1:26">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A45" s="11"/>
+      <c r="B45" s="1">
+        <v>336</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0.44122600000000001</v>
+      </c>
+      <c r="D45" s="3">
+        <v>0.441</v>
+      </c>
+      <c r="E45" s="3">
+        <v>0.27245000000000003</v>
+      </c>
+      <c r="F45" s="3">
+        <v>0.27200000000000002</v>
+      </c>
       <c r="G45" s="3">
         <v>0.438</v>
       </c>
@@ -3981,7 +4127,7 @@
         <v>0.25600000000000001</v>
       </c>
       <c r="I45" s="3">
-        <v>0.41099999999999998</v>
+        <v>0.40899999999999997</v>
       </c>
       <c r="J45" s="3">
         <v>0.27</v>
@@ -4035,7 +4181,23 @@
         <v>0.38300000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:26">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A46" s="11"/>
+      <c r="B46" s="1">
+        <v>720</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.47649900000000001</v>
+      </c>
+      <c r="D46" s="3">
+        <v>0.47599999999999998</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0.290107</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0.28999999999999998</v>
+      </c>
       <c r="G46" s="3">
         <v>0.47</v>
       </c>
@@ -4043,7 +4205,7 @@
         <v>0.27500000000000002</v>
       </c>
       <c r="I46" s="3">
-        <v>0.438</v>
+        <v>0.43099999999999999</v>
       </c>
       <c r="J46" s="3">
         <v>0.28699999999999998</v>
@@ -4097,7 +4259,35 @@
         <v>0.38200000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:26">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A47" s="11"/>
+      <c r="B47" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3">
+        <v>0.437477</v>
+      </c>
+      <c r="D47" s="3">
+        <v>0.437</v>
+      </c>
+      <c r="E47" s="3">
+        <v>0.27226899999999998</v>
+      </c>
+      <c r="F47" s="3">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="G47" s="3">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="H47" s="3">
+        <v>0.254</v>
+      </c>
+      <c r="I47" s="3">
+        <v>0.40600000000000003</v>
+      </c>
+      <c r="J47" s="3">
+        <v>27</v>
+      </c>
       <c r="K47" s="3">
         <v>0.443</v>
       </c>
@@ -4148,17 +4338,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="Q1:R1"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="Y1:Z1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="O1:P1"/>
+  <mergeCells count="19">
+    <mergeCell ref="A43:A47"/>
     <mergeCell ref="A33:A37"/>
     <mergeCell ref="A38:A42"/>
     <mergeCell ref="A3:A7"/>
@@ -4167,6 +4348,16 @@
     <mergeCell ref="A18:A22"/>
     <mergeCell ref="A23:A27"/>
     <mergeCell ref="A28:A32"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="Y1:Z1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add detailed experiment table and refresh consolidated results
- outputs/detailed-results/experiment_results_detailed.xlsx: every model
  column of the consolidated table at three decimals, truncated rather
  than rounded, for both the per-horizon and AVG rows. Best in each metric
  is bold, second best underlined, and a trailing "1 count" row totals the
  first places per model including AVG rows. Plain table, no fill colours.
- results/experiment_results.xlsx: the 3-dp display columns were TRUNC
  formulas, which biased the displayed values; they are now ROUND so the
  sheet follows round-half-up. Full-precision and baseline columns are
  unchanged, and every value still reproduces the balanced selection from
  the experiment logs.
- outputs/experiment-results-formatted/ regenerated from the corrected
  source so it no longer disagrees with it.
- Generator and verification scripts added under .spreadsheet_work/.
</commit_message>
<xml_diff>
--- a/results/experiment_results.xlsx
+++ b/results/experiment_results.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R71578c1beab64ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rcea9e19912324cc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -568,15 +568,15 @@
         <x:v>0.35903629660606384</x:v>
       </x:c>
       <x:c r="D3" s="15" t="n">
-        <x:f>TRUNC(C3,3)</x:f>
+        <x:f>ROUND(C3,3)</x:f>
         <x:v>0.359</x:v>
       </x:c>
       <x:c r="E3" s="12" t="n">
         <x:v>0.3895069360733032</x:v>
       </x:c>
       <x:c r="F3" s="17" t="n">
-        <x:f>TRUNC(E3,3)</x:f>
-        <x:v>0.389</x:v>
+        <x:f>ROUND(E3,3)</x:f>
+        <x:v>0.39</x:v>
       </x:c>
       <x:c r="G3" s="3">
         <x:v>0.374</x:v>
@@ -648,15 +648,15 @@
         <x:v>0.4111686646938324</x:v>
       </x:c>
       <x:c r="D4" s="15" t="n">
-        <x:f t="shared" ref="D4:D42" si="0">TRUNC(C4,3)</x:f>
+        <x:f t="shared" ref="D4:D42" si="0">ROUND(C4,3)</x:f>
         <x:v>0.411</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
         <x:v>0.4168122708797455</x:v>
       </x:c>
       <x:c r="F4" s="17" t="n">
-        <x:f t="shared" ref="F4:F42" si="1">TRUNC(E4,3)</x:f>
-        <x:v>0.416</x:v>
+        <x:f t="shared" ref="F4:F42" si="1">ROUND(E4,3)</x:f>
+        <x:v>0.417</x:v>
       </x:c>
       <x:c r="G4" s="3">
         <x:v>0.42699999999999999</x:v>
@@ -728,15 +728,15 @@
         <x:v>0.42646080255508423</x:v>
       </x:c>
       <x:c r="D5" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C5,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C5,3)</x:f>
         <x:v>0.426</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
         <x:v>0.43076062202453613</x:v>
       </x:c>
       <x:c r="F5" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E5,3)</x:f>
-        <x:v>0.43</x:v>
+        <x:f t="shared" si="1">ROUND(E5,3)</x:f>
+        <x:v>0.431</x:v>
       </x:c>
       <x:c r="G5" s="3">
         <x:v>0.46800000000000003</x:v>
@@ -808,15 +808,15 @@
         <x:v>0.45363208651542664</x:v>
       </x:c>
       <x:c r="D6" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C6,3)</x:f>
-        <x:v>0.453</x:v>
+        <x:f t="shared" si="0">ROUND(C6,3)</x:f>
+        <x:v>0.454</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:v>0.4546850323677063</x:v>
       </x:c>
       <x:c r="F6" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E6,3)</x:f>
-        <x:v>0.454</x:v>
+        <x:f t="shared" si="1">ROUND(E6,3)</x:f>
+        <x:v>0.455</x:v>
       </x:c>
       <x:c r="G6" s="3">
         <x:v>0.45500000000000002</x:v>
@@ -889,16 +889,16 @@
         <x:v>0.4125744625926018</x:v>
       </x:c>
       <x:c r="D7" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C7,3)</x:f>
-        <x:v>0.412</x:v>
+        <x:f t="shared" si="0">ROUND(C7,3)</x:f>
+        <x:v>0.413</x:v>
       </x:c>
       <x:c r="E7" s="13" t="n">
         <x:f>AVERAGE(E3:E6)</x:f>
         <x:v>0.4229412153363228</x:v>
       </x:c>
       <x:c r="F7" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E7,3)</x:f>
-        <x:v>0.422</x:v>
+        <x:f t="shared" si="1">ROUND(E7,3)</x:f>
+        <x:v>0.423</x:v>
       </x:c>
       <x:c r="G7" s="3" t="n">
         <x:f>AVERAGE(G3:G6)</x:f>
@@ -973,14 +973,14 @@
         <x:v>0.3014746308326721</x:v>
       </x:c>
       <x:c r="D8" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C8,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C8,3)</x:f>
         <x:v>0.301</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
         <x:v>0.3461741805076599</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E8,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E8,3)</x:f>
         <x:v>0.346</x:v>
       </x:c>
       <x:c r="G8" s="3">
@@ -1053,15 +1053,15 @@
         <x:v>0.34795844554901123</x:v>
       </x:c>
       <x:c r="D9" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C9,3)</x:f>
-        <x:v>0.347</x:v>
+        <x:f t="shared" si="0">ROUND(C9,3)</x:f>
+        <x:v>0.348</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
         <x:v>0.37466222047805786</x:v>
       </x:c>
       <x:c r="F9" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E9,3)</x:f>
-        <x:v>0.374</x:v>
+        <x:f t="shared" si="1">ROUND(E9,3)</x:f>
+        <x:v>0.375</x:v>
       </x:c>
       <x:c r="G9" s="3">
         <x:v>0.35899999999999999</x:v>
@@ -1133,14 +1133,14 @@
         <x:v>0.3766934871673584</x:v>
       </x:c>
       <x:c r="D10" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C10,3)</x:f>
-        <x:v>0.376</x:v>
+        <x:f t="shared" si="0">ROUND(C10,3)</x:f>
+        <x:v>0.377</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
         <x:v>0.39734339714050293</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E10,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E10,3)</x:f>
         <x:v>0.397</x:v>
       </x:c>
       <x:c r="G10" s="3">
@@ -1213,14 +1213,14 @@
         <x:v>0.43696802854537964</x:v>
       </x:c>
       <x:c r="D11" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C11,3)</x:f>
-        <x:v>0.436</x:v>
+        <x:f t="shared" si="0">ROUND(C11,3)</x:f>
+        <x:v>0.437</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
         <x:v>0.4312897026538849</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E11,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E11,3)</x:f>
         <x:v>0.431</x:v>
       </x:c>
       <x:c r="G11" s="3">
@@ -1294,15 +1294,15 @@
         <x:v>0.36577364802360535</x:v>
       </x:c>
       <x:c r="D12" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C12,3)</x:f>
-        <x:v>0.365</x:v>
+        <x:f t="shared" si="0">ROUND(C12,3)</x:f>
+        <x:v>0.366</x:v>
       </x:c>
       <x:c r="E12" s="13" t="n">
         <x:f>AVERAGE(E8:E11)</x:f>
         <x:v>0.3873673751950264</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E12,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E12,3)</x:f>
         <x:v>0.387</x:v>
       </x:c>
       <x:c r="G12" s="3">
@@ -1377,14 +1377,14 @@
         <x:v>0.2725314497947693</x:v>
       </x:c>
       <x:c r="D13" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C13,3)</x:f>
-        <x:v>0.272</x:v>
+        <x:f t="shared" si="0">ROUND(C13,3)</x:f>
+        <x:v>0.273</x:v>
       </x:c>
       <x:c r="E13" s="12" t="n">
         <x:v>0.33419284224510193</x:v>
       </x:c>
       <x:c r="F13" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E13,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E13,3)</x:f>
         <x:v>0.334</x:v>
       </x:c>
       <x:c r="G13" s="3">
@@ -1457,15 +1457,15 @@
         <x:v>0.35397475957870483</x:v>
       </x:c>
       <x:c r="D14" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C14,3)</x:f>
-        <x:v>0.353</x:v>
+        <x:f t="shared" si="0">ROUND(C14,3)</x:f>
+        <x:v>0.354</x:v>
       </x:c>
       <x:c r="E14" s="12" t="n">
         <x:v>0.38573458790779114</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E14,3)</x:f>
-        <x:v>0.385</x:v>
+        <x:f t="shared" si="1">ROUND(E14,3)</x:f>
+        <x:v>0.386</x:v>
       </x:c>
       <x:c r="G14" s="3">
         <x:v>0.36599999999999999</x:v>
@@ -1537,14 +1537,14 @@
         <x:v>0.3610353469848633</x:v>
       </x:c>
       <x:c r="D15" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C15,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C15,3)</x:f>
         <x:v>0.361</x:v>
       </x:c>
       <x:c r="E15" s="12" t="n">
         <x:v>0.39727529883384705</x:v>
       </x:c>
       <x:c r="F15" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E15,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E15,3)</x:f>
         <x:v>0.397</x:v>
       </x:c>
       <x:c r="G15" s="3">
@@ -1617,14 +1617,14 @@
         <x:v>0.40876638889312744</x:v>
       </x:c>
       <x:c r="D16" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C16,3)</x:f>
-        <x:v>0.408</x:v>
+        <x:f t="shared" si="0">ROUND(C16,3)</x:f>
+        <x:v>0.409</x:v>
       </x:c>
       <x:c r="E16" s="12" t="n">
         <x:v>0.43334636092185974</x:v>
       </x:c>
       <x:c r="F16" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E16,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E16,3)</x:f>
         <x:v>0.433</x:v>
       </x:c>
       <x:c r="G16" s="3">
@@ -1698,7 +1698,7 @@
         <x:v>0.3490769863128662</x:v>
       </x:c>
       <x:c r="D17" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C17,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C17,3)</x:f>
         <x:v>0.349</x:v>
       </x:c>
       <x:c r="E17" s="13" t="n">
@@ -1706,8 +1706,8 @@
         <x:v>0.38763727247714996</x:v>
       </x:c>
       <x:c r="F17" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E17,3)</x:f>
-        <x:v>0.387</x:v>
+        <x:f t="shared" si="1">ROUND(E17,3)</x:f>
+        <x:v>0.388</x:v>
       </x:c>
       <x:c r="G17" s="3">
         <x:v>0.373</x:v>
@@ -1781,15 +1781,15 @@
         <x:v>0.16781453788280487</x:v>
       </x:c>
       <x:c r="D18" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C18,3)</x:f>
-        <x:v>0.167</x:v>
+        <x:f t="shared" si="0">ROUND(C18,3)</x:f>
+        <x:v>0.168</x:v>
       </x:c>
       <x:c r="E18" s="12" t="n">
         <x:v>0.24983803927898407</x:v>
       </x:c>
       <x:c r="F18" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E18,3)</x:f>
-        <x:v>0.249</x:v>
+        <x:f t="shared" si="1">ROUND(E18,3)</x:f>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="G18" s="3">
         <x:v>0.16700000000000001</x:v>
@@ -1861,15 +1861,15 @@
         <x:v>0.23184636235237122</x:v>
       </x:c>
       <x:c r="D19" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C19,3)</x:f>
-        <x:v>0.231</x:v>
+        <x:f t="shared" si="0">ROUND(C19,3)</x:f>
+        <x:v>0.232</x:v>
       </x:c>
       <x:c r="E19" s="12" t="n">
         <x:v>0.2915283143520355</x:v>
       </x:c>
       <x:c r="F19" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E19,3)</x:f>
-        <x:v>0.291</x:v>
+        <x:f t="shared" si="1">ROUND(E19,3)</x:f>
+        <x:v>0.292</x:v>
       </x:c>
       <x:c r="G19" s="3">
         <x:v>0.23300000000000001</x:v>
@@ -1941,14 +1941,14 @@
         <x:v>0.29102447628974915</x:v>
       </x:c>
       <x:c r="D20" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C20,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C20,3)</x:f>
         <x:v>0.291</x:v>
       </x:c>
       <x:c r="E20" s="12" t="n">
         <x:v>0.332037091255188</x:v>
       </x:c>
       <x:c r="F20" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E20,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E20,3)</x:f>
         <x:v>0.332</x:v>
       </x:c>
       <x:c r="G20" s="3">
@@ -2021,15 +2021,15 @@
         <x:v>0.3846535384654999</x:v>
       </x:c>
       <x:c r="D21" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C21,3)</x:f>
-        <x:v>0.384</x:v>
+        <x:f t="shared" si="0">ROUND(C21,3)</x:f>
+        <x:v>0.385</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
         <x:v>0.38953590393066406</x:v>
       </x:c>
       <x:c r="F21" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E21,3)</x:f>
-        <x:v>0.389</x:v>
+        <x:f t="shared" si="1">ROUND(E21,3)</x:f>
+        <x:v>0.39</x:v>
       </x:c>
       <x:c r="G21" s="3">
         <x:v>0.39</x:v>
@@ -2102,16 +2102,16 @@
         <x:v>0.2688347287476063</x:v>
       </x:c>
       <x:c r="D22" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C22,3)</x:f>
-        <x:v>0.268</x:v>
+        <x:f t="shared" si="0">ROUND(C22,3)</x:f>
+        <x:v>0.269</x:v>
       </x:c>
       <x:c r="E22" s="13" t="n">
         <x:f>AVERAGE(E18:E21)</x:f>
         <x:v>0.3157348372042179</x:v>
       </x:c>
       <x:c r="F22" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E22,3)</x:f>
-        <x:v>0.315</x:v>
+        <x:f t="shared" si="1">ROUND(E22,3)</x:f>
+        <x:v>0.316</x:v>
       </x:c>
       <x:c r="G22" s="3">
         <x:v>0.27</x:v>
@@ -2185,15 +2185,15 @@
         <x:v>0.13177268207073212</x:v>
       </x:c>
       <x:c r="D23" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C23,3)</x:f>
-        <x:v>0.131</x:v>
+        <x:f t="shared" si="0">ROUND(C23,3)</x:f>
+        <x:v>0.132</x:v>
       </x:c>
       <x:c r="E23" s="12" t="n">
         <x:v>0.2266332060098648</x:v>
       </x:c>
       <x:c r="F23" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E23,3)</x:f>
-        <x:v>0.226</x:v>
+        <x:f t="shared" si="1">ROUND(E23,3)</x:f>
+        <x:v>0.227</x:v>
       </x:c>
       <x:c r="G23" s="3">
         <x:v>0.13</x:v>
@@ -2265,15 +2265,15 @@
         <x:v>0.14109523594379425</x:v>
       </x:c>
       <x:c r="D24" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C24,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C24,3)</x:f>
         <x:v>0.141</x:v>
       </x:c>
       <x:c r="E24" s="12" t="n">
         <x:v>0.23986858129501343</x:v>
       </x:c>
       <x:c r="F24" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E24,3)</x:f>
-        <x:v>0.239</x:v>
+        <x:f t="shared" si="1">ROUND(E24,3)</x:f>
+        <x:v>0.24</x:v>
       </x:c>
       <x:c r="G24" s="3">
         <x:v>0.15</x:v>
@@ -2345,15 +2345,15 @@
         <x:v>0.16397526860237122</x:v>
       </x:c>
       <x:c r="D25" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C25,3)</x:f>
-        <x:v>0.163</x:v>
+        <x:f t="shared" si="0">ROUND(C25,3)</x:f>
+        <x:v>0.164</x:v>
       </x:c>
       <x:c r="E25" s="12" t="n">
         <x:v>0.25961774587631226</x:v>
       </x:c>
       <x:c r="F25" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E25,3)</x:f>
-        <x:v>0.259</x:v>
+        <x:f t="shared" si="1">ROUND(E25,3)</x:f>
+        <x:v>0.26</x:v>
       </x:c>
       <x:c r="G25" s="3">
         <x:v>0.16500000000000001</x:v>
@@ -2425,14 +2425,14 @@
         <x:v>0.18813106417655945</x:v>
       </x:c>
       <x:c r="D26" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C26,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C26,3)</x:f>
         <x:v>0.188</x:v>
       </x:c>
       <x:c r="E26" s="12" t="n">
         <x:v>0.28333020210266113</x:v>
       </x:c>
       <x:c r="F26" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E26,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E26,3)</x:f>
         <x:v>0.283</x:v>
       </x:c>
       <x:c r="G26" s="3">
@@ -2506,7 +2506,7 @@
         <x:v>0.15624356269836426</x:v>
       </x:c>
       <x:c r="D27" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C27,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C27,3)</x:f>
         <x:v>0.156</x:v>
       </x:c>
       <x:c r="E27" s="13" t="n">
@@ -2514,7 +2514,7 @@
         <x:v>0.2523624338209629</x:v>
       </x:c>
       <x:c r="F27" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E27,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E27,3)</x:f>
         <x:v>0.252</x:v>
       </x:c>
       <x:c r="G27" s="3">
@@ -2589,14 +2589,14 @@
         <x:v>0.15067587792873383</x:v>
       </x:c>
       <x:c r="D28" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C28,3)</x:f>
-        <x:v>0.15</x:v>
+        <x:f t="shared" si="0">ROUND(C28,3)</x:f>
+        <x:v>0.151</x:v>
       </x:c>
       <x:c r="E28" s="12" t="n">
         <x:v>0.1943844109773636</x:v>
       </x:c>
       <x:c r="F28" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E28,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E28,3)</x:f>
         <x:v>0.194</x:v>
       </x:c>
       <x:c r="G28" s="3">
@@ -2669,15 +2669,15 @@
         <x:v>0.19975751638412476</x:v>
       </x:c>
       <x:c r="D29" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C29,3)</x:f>
-        <x:v>0.199</x:v>
+        <x:f t="shared" si="0">ROUND(C29,3)</x:f>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="E29" s="12" t="n">
         <x:v>0.24056372046470642</x:v>
       </x:c>
       <x:c r="F29" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E29,3)</x:f>
-        <x:v>0.24</x:v>
+        <x:f t="shared" si="1">ROUND(E29,3)</x:f>
+        <x:v>0.241</x:v>
       </x:c>
       <x:c r="G29" s="3">
         <x:v>0.20399999999999999</x:v>
@@ -2749,15 +2749,15 @@
         <x:v>0.2562653720378876</x:v>
       </x:c>
       <x:c r="D30" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C30,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C30,3)</x:f>
         <x:v>0.256</x:v>
       </x:c>
       <x:c r="E30" s="12" t="n">
         <x:v>0.28458598256111145</x:v>
       </x:c>
       <x:c r="F30" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E30,3)</x:f>
-        <x:v>0.284</x:v>
+        <x:f t="shared" si="1">ROUND(E30,3)</x:f>
+        <x:v>0.285</x:v>
       </x:c>
       <x:c r="G30" s="3">
         <x:v>0.26100000000000001</x:v>
@@ -2829,15 +2829,15 @@
         <x:v>0.33585551381111145</x:v>
       </x:c>
       <x:c r="D31" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C31,3)</x:f>
-        <x:v>0.335</x:v>
+        <x:f t="shared" si="0">ROUND(C31,3)</x:f>
+        <x:v>0.336</x:v>
       </x:c>
       <x:c r="E31" s="12" t="n">
         <x:v>0.3389362394809723</x:v>
       </x:c>
       <x:c r="F31" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E31,3)</x:f>
-        <x:v>0.338</x:v>
+        <x:f t="shared" si="1">ROUND(E31,3)</x:f>
+        <x:v>0.339</x:v>
       </x:c>
       <x:c r="G31" s="3">
         <x:v>0.34200000000000003</x:v>
@@ -2910,16 +2910,16 @@
         <x:v>0.2356385700404644</x:v>
       </x:c>
       <x:c r="D32" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C32,3)</x:f>
-        <x:v>0.235</x:v>
+        <x:f t="shared" si="0">ROUND(C32,3)</x:f>
+        <x:v>0.236</x:v>
       </x:c>
       <x:c r="E32" s="13" t="n">
         <x:f>AVERAGE(E28:E31)</x:f>
         <x:v>0.26461758837103844</x:v>
       </x:c>
       <x:c r="F32" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E32,3)</x:f>
-        <x:v>0.264</x:v>
+        <x:f t="shared" si="1">ROUND(E32,3)</x:f>
+        <x:v>0.265</x:v>
       </x:c>
       <x:c r="G32" s="3">
         <x:v>0.24</x:v>
@@ -2993,15 +2993,15 @@
         <x:v>0.16067546606063843</x:v>
       </x:c>
       <x:c r="D33" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C33,3)</x:f>
-        <x:v>0.16</x:v>
+        <x:f t="shared" si="0">ROUND(C33,3)</x:f>
+        <x:v>0.161</x:v>
       </x:c>
       <x:c r="E33" s="12" t="n">
         <x:v>0.21857710182666779</x:v>
       </x:c>
       <x:c r="F33" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E33,3)</x:f>
-        <x:v>0.218</x:v>
+        <x:f t="shared" si="1">ROUND(E33,3)</x:f>
+        <x:v>0.219</x:v>
       </x:c>
       <x:c r="G33" s="3">
         <x:v>0.16800000000000001</x:v>
@@ -3073,15 +3073,15 @@
         <x:v>0.18075653910636902</x:v>
       </x:c>
       <x:c r="D34" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C34,3)</x:f>
-        <x:v>0.18</x:v>
+        <x:f t="shared" si="0">ROUND(C34,3)</x:f>
+        <x:v>0.181</x:v>
       </x:c>
       <x:c r="E34" s="12" t="n">
         <x:v>0.24666832387447357</x:v>
       </x:c>
       <x:c r="F34" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E34,3)</x:f>
-        <x:v>0.246</x:v>
+        <x:f t="shared" si="1">ROUND(E34,3)</x:f>
+        <x:v>0.247</x:v>
       </x:c>
       <x:c r="G34" s="3">
         <x:v>0.19</x:v>
@@ -3153,14 +3153,14 @@
         <x:v>0.1906615048646927</x:v>
       </x:c>
       <x:c r="D35" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C35,3)</x:f>
-        <x:v>0.19</x:v>
+        <x:f t="shared" si="0">ROUND(C35,3)</x:f>
+        <x:v>0.191</x:v>
       </x:c>
       <x:c r="E35" s="12" t="n">
         <x:v>0.25321558117866516</x:v>
       </x:c>
       <x:c r="F35" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E35,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E35,3)</x:f>
         <x:v>0.253</x:v>
       </x:c>
       <x:c r="G35" s="3">
@@ -3233,14 +3233,14 @@
         <x:v>0.19964773952960968</x:v>
       </x:c>
       <x:c r="D36" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C36,3)</x:f>
-        <x:v>0.199</x:v>
+        <x:f t="shared" si="0">ROUND(C36,3)</x:f>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
         <x:v>0.2511758506298065</x:v>
       </x:c>
       <x:c r="F36" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E36,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E36,3)</x:f>
         <x:v>0.251</x:v>
       </x:c>
       <x:c r="G36" s="3">
@@ -3314,15 +3314,15 @@
         <x:v>0.18293531239032745</x:v>
       </x:c>
       <x:c r="D37" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C37,3)</x:f>
-        <x:v>0.182</x:v>
+        <x:f t="shared" si="0">ROUND(C37,3)</x:f>
+        <x:v>0.183</x:v>
       </x:c>
       <x:c r="E37" s="13" t="n">
         <x:f>AVERAGE(E33:E36)</x:f>
         <x:v>0.24240921437740326</x:v>
       </x:c>
       <x:c r="F37" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E37,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E37,3)</x:f>
         <x:v>0.242</x:v>
       </x:c>
       <x:c r="G37" s="3">
@@ -3397,15 +3397,15 @@
         <x:v>0.08397781848907471</x:v>
       </x:c>
       <x:c r="D38" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C38,3)</x:f>
-        <x:v>0.083</x:v>
+        <x:f t="shared" si="0">ROUND(C38,3)</x:f>
+        <x:v>0.084</x:v>
       </x:c>
       <x:c r="E38" s="12" t="n">
         <x:v>0.20274776220321655</x:v>
       </x:c>
       <x:c r="F38" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E38,3)</x:f>
-        <x:v>0.202</x:v>
+        <x:f t="shared" si="1">ROUND(E38,3)</x:f>
+        <x:v>0.203</x:v>
       </x:c>
       <x:c r="G38" s="3">
         <x:v>8.3000000000000004E-2</x:v>
@@ -3471,14 +3471,14 @@
         <x:v>0.17626334726810455</x:v>
       </x:c>
       <x:c r="D39" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C39,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C39,3)</x:f>
         <x:v>0.176</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
         <x:v>0.29905030131340027</x:v>
       </x:c>
       <x:c r="F39" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E39,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E39,3)</x:f>
         <x:v>0.299</x:v>
       </x:c>
       <x:c r="G39" s="3">
@@ -3545,15 +3545,15 @@
         <x:v>0.3257855474948883</x:v>
       </x:c>
       <x:c r="D40" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C40,3)</x:f>
-        <x:v>0.325</x:v>
+        <x:f t="shared" si="0">ROUND(C40,3)</x:f>
+        <x:v>0.326</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
         <x:v>0.4118848443031311</x:v>
       </x:c>
       <x:c r="F40" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E40,3)</x:f>
-        <x:v>0.411</x:v>
+        <x:f t="shared" si="1">ROUND(E40,3)</x:f>
+        <x:v>0.412</x:v>
       </x:c>
       <x:c r="G40" s="3">
         <x:v>0.33400000000000002</x:v>
@@ -3619,14 +3619,14 @@
         <x:v>0.7918639183044434</x:v>
       </x:c>
       <x:c r="D41" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C41,3)</x:f>
-        <x:v>0.791</x:v>
+        <x:f t="shared" si="0">ROUND(C41,3)</x:f>
+        <x:v>0.792</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
         <x:v>0.6723057627677917</x:v>
       </x:c>
       <x:c r="F41" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E41,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E41,3)</x:f>
         <x:v>0.672</x:v>
       </x:c>
       <x:c r="G41" s="3">
@@ -3694,7 +3694,7 @@
         <x:v>0.34447265788912773</x:v>
       </x:c>
       <x:c r="D42" s="15" t="n">
-        <x:f t="shared" si="0">TRUNC(C42,3)</x:f>
+        <x:f t="shared" si="0">ROUND(C42,3)</x:f>
         <x:v>0.344</x:v>
       </x:c>
       <x:c r="E42" s="13" t="n">
@@ -3702,7 +3702,7 @@
         <x:v>0.3964971676468849</x:v>
       </x:c>
       <x:c r="F42" s="17" t="n">
-        <x:f t="shared" si="1">TRUNC(E42,3)</x:f>
+        <x:f t="shared" si="1">ROUND(E42,3)</x:f>
         <x:v>0.396</x:v>
       </x:c>
       <x:c r="G42" s="3">
@@ -3771,14 +3771,14 @@
         <x:v>0.4104566276073456</x:v>
       </x:c>
       <x:c r="D43" s="16" t="n">
-        <x:f>TRUNC(C43,3)</x:f>
+        <x:f>ROUND(C43,3)</x:f>
         <x:v>0.41</x:v>
       </x:c>
       <x:c r="E43" s="14" t="n">
         <x:v>0.2550795376300812</x:v>
       </x:c>
       <x:c r="F43" s="16" t="n">
-        <x:f>TRUNC(E43,3)</x:f>
+        <x:f>ROUND(E43,3)</x:f>
         <x:v>0.255</x:v>
       </x:c>
       <x:c r="G43" s="3">
@@ -3851,14 +3851,14 @@
         <x:v>0.4242447018623352</x:v>
       </x:c>
       <x:c r="D44" s="16" t="n">
-        <x:f>TRUNC(C44,3)</x:f>
+        <x:f>ROUND(C44,3)</x:f>
         <x:v>0.424</x:v>
       </x:c>
       <x:c r="E44" s="14" t="n">
         <x:v>0.26533040404319763</x:v>
       </x:c>
       <x:c r="F44" s="16" t="n">
-        <x:f>TRUNC(E44,3)</x:f>
+        <x:f>ROUND(E44,3)</x:f>
         <x:v>0.265</x:v>
       </x:c>
       <x:c r="G44" s="3">
@@ -3931,14 +3931,14 @@
         <x:v>0.4412255585193634</x:v>
       </x:c>
       <x:c r="D45" s="16" t="n">
-        <x:f>TRUNC(C45,3)</x:f>
+        <x:f>ROUND(C45,3)</x:f>
         <x:v>0.441</x:v>
       </x:c>
       <x:c r="E45" s="14" t="n">
         <x:v>0.2724500596523285</x:v>
       </x:c>
       <x:c r="F45" s="16" t="n">
-        <x:f>TRUNC(E45,3)</x:f>
+        <x:f>ROUND(E45,3)</x:f>
         <x:v>0.272</x:v>
       </x:c>
       <x:c r="G45" s="3">
@@ -4011,14 +4011,14 @@
         <x:v>0.47649940848350525</x:v>
       </x:c>
       <x:c r="D46" s="16" t="n">
-        <x:f>TRUNC(C46,3)</x:f>
+        <x:f>ROUND(C46,3)</x:f>
         <x:v>0.476</x:v>
       </x:c>
       <x:c r="E46" s="14" t="n">
         <x:v>0.29010656476020813</x:v>
       </x:c>
       <x:c r="F46" s="16" t="n">
-        <x:f>TRUNC(E46,3)</x:f>
+        <x:f>ROUND(E46,3)</x:f>
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="G46" s="3">
@@ -4092,7 +4092,7 @@
         <x:v>0.43810657411813736</x:v>
       </x:c>
       <x:c r="D47" s="16" t="n">
-        <x:f>TRUNC(C47,3)</x:f>
+        <x:f>ROUND(C47,3)</x:f>
         <x:v>0.438</x:v>
       </x:c>
       <x:c r="E47" s="14" t="n">
@@ -4100,8 +4100,8 @@
         <x:v>0.27074164152145386</x:v>
       </x:c>
       <x:c r="F47" s="16" t="n">
-        <x:f>TRUNC(E47,3)</x:f>
-        <x:v>0.27</x:v>
+        <x:f>ROUND(E47,3)</x:f>
+        <x:v>0.271</x:v>
       </x:c>
       <x:c r="G47" s="3">
         <x:v>0.43099999999999999</x:v>

</xml_diff>